<commit_message>
map-bf-9 results with pd and hopa baselines
</commit_message>
<xml_diff>
--- a/workspace/framework_paper/map-bf/map-bf-9/map-bf-9_schedulables.xlsx
+++ b/workspace/framework_paper/map-bf/map-bf-9/map-bf-9_schedulables.xlsx
@@ -413,21 +413,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" t="inlineStr">
         <is>
+          <t>pd</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>hopa</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>gdpa-100</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>gdpa-200</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>bf</t>
         </is>
@@ -446,6 +456,12 @@
       <c r="D2" t="n">
         <v>25</v>
       </c>
+      <c r="E2" t="n">
+        <v>25</v>
+      </c>
+      <c r="F2" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -460,6 +476,12 @@
       <c r="D3" t="n">
         <v>25</v>
       </c>
+      <c r="E3" t="n">
+        <v>25</v>
+      </c>
+      <c r="F3" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -474,18 +496,30 @@
       <c r="D4" t="n">
         <v>25</v>
       </c>
+      <c r="E4" t="n">
+        <v>25</v>
+      </c>
+      <c r="F4" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
         <v>0.5631578947368421</v>
       </c>
       <c r="B5" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C5" t="n">
         <v>25</v>
       </c>
       <c r="D5" t="n">
+        <v>25</v>
+      </c>
+      <c r="E5" t="n">
+        <v>25</v>
+      </c>
+      <c r="F5" t="n">
         <v>25</v>
       </c>
     </row>
@@ -494,12 +528,18 @@
         <v>0.5842105263157895</v>
       </c>
       <c r="B6" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C6" t="n">
         <v>25</v>
       </c>
       <c r="D6" t="n">
+        <v>25</v>
+      </c>
+      <c r="E6" t="n">
+        <v>25</v>
+      </c>
+      <c r="F6" t="n">
         <v>25</v>
       </c>
     </row>
@@ -508,12 +548,18 @@
         <v>0.6052631578947368</v>
       </c>
       <c r="B7" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C7" t="n">
         <v>25</v>
       </c>
       <c r="D7" t="n">
+        <v>25</v>
+      </c>
+      <c r="E7" t="n">
+        <v>25</v>
+      </c>
+      <c r="F7" t="n">
         <v>25</v>
       </c>
     </row>
@@ -522,12 +568,18 @@
         <v>0.6263157894736842</v>
       </c>
       <c r="B8" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C8" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D8" t="n">
+        <v>25</v>
+      </c>
+      <c r="E8" t="n">
+        <v>25</v>
+      </c>
+      <c r="F8" t="n">
         <v>25</v>
       </c>
     </row>
@@ -536,12 +588,18 @@
         <v>0.6473684210526316</v>
       </c>
       <c r="B9" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="C9" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="D9" t="n">
+        <v>25</v>
+      </c>
+      <c r="E9" t="n">
+        <v>25</v>
+      </c>
+      <c r="F9" t="n">
         <v>25</v>
       </c>
     </row>
@@ -550,12 +608,18 @@
         <v>0.6684210526315789</v>
       </c>
       <c r="B10" t="n">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="C10" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D10" t="n">
+        <v>25</v>
+      </c>
+      <c r="E10" t="n">
+        <v>25</v>
+      </c>
+      <c r="F10" t="n">
         <v>25</v>
       </c>
     </row>
@@ -564,12 +628,18 @@
         <v>0.6894736842105263</v>
       </c>
       <c r="B11" t="n">
+        <v>11</v>
+      </c>
+      <c r="C11" t="n">
+        <v>20</v>
+      </c>
+      <c r="D11" t="n">
         <v>24</v>
       </c>
-      <c r="C11" t="n">
-        <v>25</v>
-      </c>
-      <c r="D11" t="n">
+      <c r="E11" t="n">
+        <v>25</v>
+      </c>
+      <c r="F11" t="n">
         <v>25</v>
       </c>
     </row>
@@ -578,12 +648,18 @@
         <v>0.7105263157894737</v>
       </c>
       <c r="B12" t="n">
+        <v>8</v>
+      </c>
+      <c r="C12" t="n">
+        <v>15</v>
+      </c>
+      <c r="D12" t="n">
         <v>23</v>
       </c>
-      <c r="C12" t="n">
+      <c r="E12" t="n">
         <v>23</v>
       </c>
-      <c r="D12" t="n">
+      <c r="F12" t="n">
         <v>25</v>
       </c>
     </row>
@@ -592,12 +668,18 @@
         <v>0.7315789473684211</v>
       </c>
       <c r="B13" t="n">
+        <v>6</v>
+      </c>
+      <c r="C13" t="n">
+        <v>7</v>
+      </c>
+      <c r="D13" t="n">
         <v>18</v>
       </c>
-      <c r="C13" t="n">
+      <c r="E13" t="n">
         <v>18</v>
       </c>
-      <c r="D13" t="n">
+      <c r="F13" t="n">
         <v>24</v>
       </c>
     </row>
@@ -606,12 +688,18 @@
         <v>0.7526315789473684</v>
       </c>
       <c r="B14" t="n">
+        <v>5</v>
+      </c>
+      <c r="C14" t="n">
+        <v>5</v>
+      </c>
+      <c r="D14" t="n">
         <v>18</v>
       </c>
-      <c r="C14" t="n">
+      <c r="E14" t="n">
         <v>18</v>
       </c>
-      <c r="D14" t="n">
+      <c r="F14" t="n">
         <v>23</v>
       </c>
     </row>
@@ -620,12 +708,18 @@
         <v>0.7736842105263158</v>
       </c>
       <c r="B15" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" t="n">
         <v>16</v>
       </c>
-      <c r="C15" t="n">
+      <c r="E15" t="n">
         <v>17</v>
       </c>
-      <c r="D15" t="n">
+      <c r="F15" t="n">
         <v>23</v>
       </c>
     </row>
@@ -634,12 +728,18 @@
         <v>0.7947368421052632</v>
       </c>
       <c r="B16" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" t="n">
         <v>18</v>
       </c>
-      <c r="C16" t="n">
+      <c r="E16" t="n">
         <v>18</v>
       </c>
-      <c r="D16" t="n">
+      <c r="F16" t="n">
         <v>22</v>
       </c>
     </row>
@@ -648,12 +748,18 @@
         <v>0.8157894736842105</v>
       </c>
       <c r="B17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" t="n">
         <v>16</v>
       </c>
-      <c r="C17" t="n">
+      <c r="E17" t="n">
         <v>16</v>
       </c>
-      <c r="D17" t="n">
+      <c r="F17" t="n">
         <v>20</v>
       </c>
     </row>
@@ -662,12 +768,18 @@
         <v>0.8368421052631578</v>
       </c>
       <c r="B18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" t="n">
         <v>12</v>
       </c>
-      <c r="C18" t="n">
+      <c r="E18" t="n">
         <v>12</v>
       </c>
-      <c r="D18" t="n">
+      <c r="F18" t="n">
         <v>20</v>
       </c>
     </row>
@@ -676,12 +788,18 @@
         <v>0.8578947368421053</v>
       </c>
       <c r="B19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" t="n">
         <v>10</v>
       </c>
-      <c r="C19" t="n">
+      <c r="E19" t="n">
         <v>12</v>
       </c>
-      <c r="D19" t="n">
+      <c r="F19" t="n">
         <v>19</v>
       </c>
     </row>
@@ -690,12 +808,18 @@
         <v>0.8789473684210527</v>
       </c>
       <c r="B20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" t="n">
         <v>9</v>
       </c>
-      <c r="C20" t="n">
+      <c r="E20" t="n">
         <v>10</v>
       </c>
-      <c r="D20" t="n">
+      <c r="F20" t="n">
         <v>17</v>
       </c>
     </row>
@@ -704,12 +828,18 @@
         <v>0.9</v>
       </c>
       <c r="B21" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" t="n">
         <v>8</v>
       </c>
-      <c r="C21" t="n">
+      <c r="E21" t="n">
         <v>8</v>
       </c>
-      <c r="D21" t="n">
+      <c r="F21" t="n">
         <v>16</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add gdpa-prio column to map-bf-9 results
</commit_message>
<xml_diff>
--- a/workspace/framework_paper/map-bf/map-bf-9/map-bf-9_schedulables.xlsx
+++ b/workspace/framework_paper/map-bf/map-bf-9/map-bf-9_schedulables.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -429,15 +429,20 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>gdpa-prio</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>gdpa-100</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>gdpa-200</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>bf</t>
         </is>
@@ -462,6 +467,9 @@
       <c r="F2" t="n">
         <v>25</v>
       </c>
+      <c r="G2" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -482,6 +490,9 @@
       <c r="F3" t="n">
         <v>25</v>
       </c>
+      <c r="G3" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -502,6 +513,9 @@
       <c r="F4" t="n">
         <v>25</v>
       </c>
+      <c r="G4" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -522,6 +536,9 @@
       <c r="F5" t="n">
         <v>25</v>
       </c>
+      <c r="G5" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -542,6 +559,9 @@
       <c r="F6" t="n">
         <v>25</v>
       </c>
+      <c r="G6" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -562,6 +582,9 @@
       <c r="F7" t="n">
         <v>25</v>
       </c>
+      <c r="G7" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -582,6 +605,9 @@
       <c r="F8" t="n">
         <v>25</v>
       </c>
+      <c r="G8" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -594,12 +620,15 @@
         <v>22</v>
       </c>
       <c r="D9" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E9" t="n">
         <v>25</v>
       </c>
       <c r="F9" t="n">
+        <v>25</v>
+      </c>
+      <c r="G9" t="n">
         <v>25</v>
       </c>
     </row>
@@ -614,12 +643,15 @@
         <v>21</v>
       </c>
       <c r="D10" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="E10" t="n">
         <v>25</v>
       </c>
       <c r="F10" t="n">
+        <v>25</v>
+      </c>
+      <c r="G10" t="n">
         <v>25</v>
       </c>
     </row>
@@ -634,12 +666,15 @@
         <v>20</v>
       </c>
       <c r="D11" t="n">
+        <v>20</v>
+      </c>
+      <c r="E11" t="n">
         <v>24</v>
       </c>
-      <c r="E11" t="n">
-        <v>25</v>
-      </c>
       <c r="F11" t="n">
+        <v>25</v>
+      </c>
+      <c r="G11" t="n">
         <v>25</v>
       </c>
     </row>
@@ -654,12 +689,15 @@
         <v>15</v>
       </c>
       <c r="D12" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="E12" t="n">
         <v>23</v>
       </c>
       <c r="F12" t="n">
+        <v>23</v>
+      </c>
+      <c r="G12" t="n">
         <v>25</v>
       </c>
     </row>
@@ -674,12 +712,15 @@
         <v>7</v>
       </c>
       <c r="D13" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="E13" t="n">
         <v>18</v>
       </c>
       <c r="F13" t="n">
+        <v>18</v>
+      </c>
+      <c r="G13" t="n">
         <v>24</v>
       </c>
     </row>
@@ -694,12 +735,15 @@
         <v>5</v>
       </c>
       <c r="D14" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="E14" t="n">
         <v>18</v>
       </c>
       <c r="F14" t="n">
+        <v>18</v>
+      </c>
+      <c r="G14" t="n">
         <v>23</v>
       </c>
     </row>
@@ -714,12 +758,15 @@
         <v>1</v>
       </c>
       <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="n">
         <v>16</v>
       </c>
-      <c r="E15" t="n">
+      <c r="F15" t="n">
         <v>17</v>
       </c>
-      <c r="F15" t="n">
+      <c r="G15" t="n">
         <v>23</v>
       </c>
     </row>
@@ -734,12 +781,15 @@
         <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="E16" t="n">
         <v>18</v>
       </c>
       <c r="F16" t="n">
+        <v>18</v>
+      </c>
+      <c r="G16" t="n">
         <v>22</v>
       </c>
     </row>
@@ -754,12 +804,15 @@
         <v>0</v>
       </c>
       <c r="D17" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="E17" t="n">
         <v>16</v>
       </c>
       <c r="F17" t="n">
+        <v>16</v>
+      </c>
+      <c r="G17" t="n">
         <v>20</v>
       </c>
     </row>
@@ -774,12 +827,15 @@
         <v>0</v>
       </c>
       <c r="D18" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="E18" t="n">
         <v>12</v>
       </c>
       <c r="F18" t="n">
+        <v>12</v>
+      </c>
+      <c r="G18" t="n">
         <v>20</v>
       </c>
     </row>
@@ -794,12 +850,15 @@
         <v>0</v>
       </c>
       <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
         <v>10</v>
       </c>
-      <c r="E19" t="n">
+      <c r="F19" t="n">
         <v>12</v>
       </c>
-      <c r="F19" t="n">
+      <c r="G19" t="n">
         <v>19</v>
       </c>
     </row>
@@ -814,12 +873,15 @@
         <v>0</v>
       </c>
       <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="n">
         <v>9</v>
       </c>
-      <c r="E20" t="n">
+      <c r="F20" t="n">
         <v>10</v>
       </c>
-      <c r="F20" t="n">
+      <c r="G20" t="n">
         <v>17</v>
       </c>
     </row>
@@ -834,12 +896,15 @@
         <v>0</v>
       </c>
       <c r="D21" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="E21" t="n">
         <v>8</v>
       </c>
       <c r="F21" t="n">
+        <v>8</v>
+      </c>
+      <c r="G21" t="n">
         <v>16</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add gdpa-ms column to map-bf-9 results (451/500)
</commit_message>
<xml_diff>
--- a/workspace/framework_paper/map-bf/map-bf-9/map-bf-9_schedulables.xlsx
+++ b/workspace/framework_paper/map-bf/map-bf-9/map-bf-9_schedulables.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,6 +444,11 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>gdpa-ms</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>bf</t>
         </is>
       </c>
@@ -470,6 +475,9 @@
       <c r="G2" t="n">
         <v>25</v>
       </c>
+      <c r="H2" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -493,6 +501,9 @@
       <c r="G3" t="n">
         <v>25</v>
       </c>
+      <c r="H3" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -516,6 +527,9 @@
       <c r="G4" t="n">
         <v>25</v>
       </c>
+      <c r="H4" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -539,6 +553,9 @@
       <c r="G5" t="n">
         <v>25</v>
       </c>
+      <c r="H5" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -562,6 +579,9 @@
       <c r="G6" t="n">
         <v>25</v>
       </c>
+      <c r="H6" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -585,6 +605,9 @@
       <c r="G7" t="n">
         <v>25</v>
       </c>
+      <c r="H7" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -608,6 +631,9 @@
       <c r="G8" t="n">
         <v>25</v>
       </c>
+      <c r="H8" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -631,6 +657,9 @@
       <c r="G9" t="n">
         <v>25</v>
       </c>
+      <c r="H9" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -654,6 +683,9 @@
       <c r="G10" t="n">
         <v>25</v>
       </c>
+      <c r="H10" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -677,6 +709,9 @@
       <c r="G11" t="n">
         <v>25</v>
       </c>
+      <c r="H11" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -700,6 +735,9 @@
       <c r="G12" t="n">
         <v>25</v>
       </c>
+      <c r="H12" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -723,6 +761,9 @@
       <c r="G13" t="n">
         <v>24</v>
       </c>
+      <c r="H13" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -746,6 +787,9 @@
       <c r="G14" t="n">
         <v>23</v>
       </c>
+      <c r="H14" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -769,6 +813,9 @@
       <c r="G15" t="n">
         <v>23</v>
       </c>
+      <c r="H15" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -790,6 +837,9 @@
         <v>18</v>
       </c>
       <c r="G16" t="n">
+        <v>21</v>
+      </c>
+      <c r="H16" t="n">
         <v>22</v>
       </c>
     </row>
@@ -815,6 +865,9 @@
       <c r="G17" t="n">
         <v>20</v>
       </c>
+      <c r="H17" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -836,6 +889,9 @@
         <v>12</v>
       </c>
       <c r="G18" t="n">
+        <v>18</v>
+      </c>
+      <c r="H18" t="n">
         <v>20</v>
       </c>
     </row>
@@ -859,6 +915,9 @@
         <v>12</v>
       </c>
       <c r="G19" t="n">
+        <v>18</v>
+      </c>
+      <c r="H19" t="n">
         <v>19</v>
       </c>
     </row>
@@ -882,6 +941,9 @@
         <v>10</v>
       </c>
       <c r="G20" t="n">
+        <v>15</v>
+      </c>
+      <c r="H20" t="n">
         <v>17</v>
       </c>
     </row>
@@ -905,6 +967,9 @@
         <v>8</v>
       </c>
       <c r="G21" t="n">
+        <v>14</v>
+      </c>
+      <c r="H21" t="n">
         <v>16</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update map-bf results: bounded multi-start gdpa-100/200/500 (453/500 vs bf 459)
</commit_message>
<xml_diff>
--- a/workspace/framework_paper/map-bf/map-bf-9/map-bf-9_schedulables.xlsx
+++ b/workspace/framework_paper/map-bf/map-bf-9/map-bf-9_schedulables.xlsx
@@ -444,7 +444,7 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>gdpa-ms</t>
+          <t>gdpa-500</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
@@ -701,7 +701,7 @@
         <v>20</v>
       </c>
       <c r="E11" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F11" t="n">
         <v>25</v>
@@ -727,10 +727,10 @@
         <v>15</v>
       </c>
       <c r="E12" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F12" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G12" t="n">
         <v>25</v>
@@ -753,13 +753,13 @@
         <v>9</v>
       </c>
       <c r="E13" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F13" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="G13" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H13" t="n">
         <v>24</v>
@@ -779,10 +779,10 @@
         <v>5</v>
       </c>
       <c r="E14" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F14" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="G14" t="n">
         <v>23</v>
@@ -805,13 +805,13 @@
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="F15" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="G15" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H15" t="n">
         <v>23</v>
@@ -831,10 +831,10 @@
         <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F16" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="G16" t="n">
         <v>21</v>
@@ -857,10 +857,10 @@
         <v>0</v>
       </c>
       <c r="E17" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F17" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G17" t="n">
         <v>20</v>
@@ -883,13 +883,13 @@
         <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="F18" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="G18" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H18" t="n">
         <v>20</v>
@@ -909,13 +909,13 @@
         <v>0</v>
       </c>
       <c r="E19" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F19" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="G19" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H19" t="n">
         <v>19</v>
@@ -935,13 +935,13 @@
         <v>0</v>
       </c>
       <c r="E20" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F20" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G20" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H20" t="n">
         <v>17</v>
@@ -961,10 +961,10 @@
         <v>0</v>
       </c>
       <c r="E21" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F21" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G21" t="n">
         <v>14</v>

</xml_diff>

<commit_message>
add bf-seq column to map-bf-9 results (matches bf: 459/500)
</commit_message>
<xml_diff>
--- a/workspace/framework_paper/map-bf/map-bf-9/map-bf-9_schedulables.xlsx
+++ b/workspace/framework_paper/map-bf/map-bf-9/map-bf-9_schedulables.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,6 +452,11 @@
           <t>bf</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>bf-seq</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -478,6 +483,9 @@
       <c r="H2" t="n">
         <v>25</v>
       </c>
+      <c r="I2" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -504,6 +512,9 @@
       <c r="H3" t="n">
         <v>25</v>
       </c>
+      <c r="I3" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -530,6 +541,9 @@
       <c r="H4" t="n">
         <v>25</v>
       </c>
+      <c r="I4" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -556,6 +570,9 @@
       <c r="H5" t="n">
         <v>25</v>
       </c>
+      <c r="I5" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -582,6 +599,9 @@
       <c r="H6" t="n">
         <v>25</v>
       </c>
+      <c r="I6" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -608,6 +628,9 @@
       <c r="H7" t="n">
         <v>25</v>
       </c>
+      <c r="I7" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -634,6 +657,9 @@
       <c r="H8" t="n">
         <v>25</v>
       </c>
+      <c r="I8" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -660,6 +686,9 @@
       <c r="H9" t="n">
         <v>25</v>
       </c>
+      <c r="I9" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -686,6 +715,9 @@
       <c r="H10" t="n">
         <v>25</v>
       </c>
+      <c r="I10" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -712,6 +744,9 @@
       <c r="H11" t="n">
         <v>25</v>
       </c>
+      <c r="I11" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -738,6 +773,9 @@
       <c r="H12" t="n">
         <v>25</v>
       </c>
+      <c r="I12" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -764,6 +802,9 @@
       <c r="H13" t="n">
         <v>24</v>
       </c>
+      <c r="I13" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -790,6 +831,9 @@
       <c r="H14" t="n">
         <v>23</v>
       </c>
+      <c r="I14" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -816,6 +860,9 @@
       <c r="H15" t="n">
         <v>23</v>
       </c>
+      <c r="I15" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -842,6 +889,9 @@
       <c r="H16" t="n">
         <v>22</v>
       </c>
+      <c r="I16" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -868,6 +918,9 @@
       <c r="H17" t="n">
         <v>20</v>
       </c>
+      <c r="I17" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -894,6 +947,9 @@
       <c r="H18" t="n">
         <v>20</v>
       </c>
+      <c r="I18" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -920,6 +976,9 @@
       <c r="H19" t="n">
         <v>19</v>
       </c>
+      <c r="I19" t="n">
+        <v>19</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -946,6 +1005,9 @@
       <c r="H20" t="n">
         <v>17</v>
       </c>
+      <c r="I20" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -970,6 +1032,9 @@
         <v>14</v>
       </c>
       <c r="H21" t="n">
+        <v>16</v>
+      </c>
+      <c r="I21" t="n">
         <v>16</v>
       </c>
     </row>

</xml_diff>